<commit_message>
sei interpretazioni incoerenti con il riferimento; controllo sulle sorgenti (T-84, D-022)
Quattro correzioni (vicenza, Tivoli/Càrsoli, piazza Verdi) e due
doppioni eliminati (QP 294). audit_alignment.py confronta luogo
dell'interpretazione e luogo del riferimento nei TSV; IQ11 informativa.
ABox 16.045 -> 16.029, full 17.203 -> 17.187, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/SpatialInterpretations.xlsx
+++ b/data/source/xlsx/SpatialInterpretations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P963"/>
+  <dimension ref="A1:P961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12904,7 +12904,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t xml:space="preserve">vicenza </t>
+          <t>vicenza</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -16192,7 +16192,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>banca_ditalia</t>
+          <t>piazza_verdi</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -27788,7 +27788,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>ref_00522</t>
+          <t>ref_00523</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>ref_00523</t>
+          <t>ref_00522</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -36645,7 +36645,7 @@
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t>interp_00858</t>
+          <t>interp_00860</t>
         </is>
       </c>
       <c r="B859" t="inlineStr">
@@ -36655,7 +36655,7 @@
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>marino</t>
+          <t>tenenza_carabinieri_marino</t>
         </is>
       </c>
       <c r="D859" t="inlineStr">
@@ -36665,34 +36665,39 @@
       </c>
       <c r="E859" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G859" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>interp_00859</t>
+          <t>interp_00861</t>
         </is>
       </c>
       <c r="B860" t="inlineStr">
         <is>
-          <t>ref_00684</t>
+          <t>ref_00683</t>
         </is>
       </c>
       <c r="C860" t="inlineStr">
         <is>
-          <t>marino</t>
+          <t>tenenza_carabinieri_marino</t>
         </is>
       </c>
       <c r="D860" t="inlineStr">
@@ -36702,24 +36707,29 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F860" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G860" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr">
         <is>
-          <t>interp_00860</t>
+          <t>interp_00862</t>
         </is>
       </c>
       <c r="B861" t="inlineStr">
@@ -36739,7 +36749,7 @@
       </c>
       <c r="E861" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="F861" t="inlineStr">
@@ -36761,91 +36771,81 @@
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>interp_00861</t>
+          <t>interp_00863</t>
         </is>
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>ref_00683</t>
+          <t>ref_00684</t>
         </is>
       </c>
       <c r="C862" t="inlineStr">
         <is>
-          <t>tenenza_carabinieri_marino</t>
+          <t>via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="D862" t="inlineStr">
         <is>
-          <t>gaz_marino</t>
+          <t>gaz_via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="E862" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="F862" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G862" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H862" t="inlineStr">
-        <is>
-          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">
         <is>
-          <t>interp_00862</t>
+          <t>interp_00864</t>
         </is>
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>ref_00683</t>
+          <t>ref_00684</t>
         </is>
       </c>
       <c r="C863" t="inlineStr">
         <is>
-          <t>tenenza_carabinieri_marino</t>
+          <t>via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="D863" t="inlineStr">
         <is>
-          <t>gaz_marino</t>
+          <t>gaz_via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="E863" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F863" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G863" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H863" t="inlineStr">
-        <is>
-          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>interp_00863</t>
+          <t>interp_00865</t>
         </is>
       </c>
       <c r="B864" t="inlineStr">
@@ -36865,7 +36865,7 @@
       </c>
       <c r="E864" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="F864" t="inlineStr">
@@ -36882,32 +36882,32 @@
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>interp_00864</t>
+          <t>interp_00866</t>
         </is>
       </c>
       <c r="B865" t="inlineStr">
         <is>
-          <t>ref_00684</t>
+          <t>ref_00685</t>
         </is>
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>via_massimo_dazeglio</t>
+          <t>due_santi</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
         <is>
-          <t>gaz_via_massimo_dazeglio</t>
+          <t>gaz_due_santi</t>
         </is>
       </c>
       <c r="E865" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>pestalozzi</t>
         </is>
       </c>
       <c r="F865" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G865" t="inlineStr">
@@ -36919,123 +36919,123 @@
     <row r="866">
       <c r="A866" t="inlineStr">
         <is>
-          <t>interp_00865</t>
+          <t>interp_00867</t>
         </is>
       </c>
       <c r="B866" t="inlineStr">
         <is>
-          <t>ref_00684</t>
+          <t>ref_00686</t>
         </is>
       </c>
       <c r="C866" t="inlineStr">
         <is>
-          <t>via_massimo_dazeglio</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
         <is>
-          <t>gaz_via_massimo_dazeglio</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F866" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G866" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>relative</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="867">
       <c r="A867" t="inlineStr">
         <is>
-          <t>interp_00866</t>
+          <t>interp_00868</t>
         </is>
       </c>
       <c r="B867" t="inlineStr">
         <is>
-          <t>ref_00685</t>
+          <t>ref_00687</t>
         </is>
       </c>
       <c r="C867" t="inlineStr">
         <is>
-          <t>due_santi</t>
+          <t>via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
         <is>
-          <t>gaz_due_santi</t>
+          <t>gaz_via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="E867" t="inlineStr">
         <is>
-          <t>pestalozzi</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F867" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G867" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>relative</t>
         </is>
       </c>
     </row>
     <row r="868">
       <c r="A868" t="inlineStr">
         <is>
-          <t>interp_00867</t>
+          <t>interp_00869</t>
         </is>
       </c>
       <c r="B868" t="inlineStr">
         <is>
-          <t>ref_00686</t>
+          <t>ref_00687</t>
         </is>
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_via_massimo_dazeglio</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="F868" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G868" t="inlineStr">
         <is>
           <t>relative</t>
-        </is>
-      </c>
-      <c r="H868" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="869">
       <c r="A869" t="inlineStr">
         <is>
-          <t>interp_00868</t>
+          <t>interp_00870</t>
         </is>
       </c>
       <c r="B869" t="inlineStr">
@@ -37055,7 +37055,7 @@
       </c>
       <c r="E869" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="F869" t="inlineStr">
@@ -37072,7 +37072,7 @@
     <row r="870">
       <c r="A870" t="inlineStr">
         <is>
-          <t>interp_00869</t>
+          <t>interp_00871</t>
         </is>
       </c>
       <c r="B870" t="inlineStr">
@@ -37092,7 +37092,7 @@
       </c>
       <c r="E870" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="F870" t="inlineStr">
@@ -37109,81 +37109,87 @@
     <row r="871">
       <c r="A871" t="inlineStr">
         <is>
-          <t>interp_00870</t>
+          <t>interp_00872</t>
         </is>
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>ref_00687</t>
+          <t>ref_00688</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
         <is>
-          <t>via_massimo_dazeglio</t>
+          <t>torraccio</t>
         </is>
       </c>
       <c r="D871" t="inlineStr">
         <is>
-          <t>gaz_via_massimo_dazeglio</t>
+          <t>gaz_torraccio</t>
         </is>
       </c>
       <c r="E871" t="inlineStr">
         <is>
-          <t>autista_questura</t>
-        </is>
-      </c>
-      <c r="F871" t="inlineStr">
-        <is>
-          <t>marker</t>
-        </is>
-      </c>
-      <c r="G871" t="inlineStr">
-        <is>
-          <t>relative</t>
-        </is>
+          <t>ingravallo</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>routenode</t>
+        </is>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>tragitto_torraccio_ponte_divino_amore</t>
+        </is>
+      </c>
+      <c r="K871" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>interp_00871</t>
+          <t>interp_00873</t>
         </is>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>ref_00687</t>
+          <t>ref_00688</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>via_massimo_dazeglio</t>
+          <t>torraccio</t>
         </is>
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>gaz_via_massimo_dazeglio</t>
+          <t>gaz_torraccio</t>
         </is>
       </c>
       <c r="E872" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
-        </is>
-      </c>
-      <c r="F872" t="inlineStr">
-        <is>
-          <t>marker</t>
-        </is>
-      </c>
-      <c r="G872" t="inlineStr">
-        <is>
-          <t>relative</t>
-        </is>
+          <t>maresciallo_di_pietrantonio</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>routenode</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>tragitto_torraccio_ponte_divino_amore</t>
+        </is>
+      </c>
+      <c r="K872" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>interp_00872</t>
+          <t>interp_00874</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
@@ -37203,7 +37209,7 @@
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I873" t="inlineStr">
@@ -37223,7 +37229,7 @@
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>interp_00873</t>
+          <t>interp_00875</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
@@ -37243,7 +37249,7 @@
       </c>
       <c r="E874" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I874" t="inlineStr">
@@ -37263,27 +37269,27 @@
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>interp_00874</t>
+          <t>interp_00876</t>
         </is>
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>ref_00688</t>
+          <t>ref_00689</t>
         </is>
       </c>
       <c r="C875" t="inlineStr">
         <is>
-          <t>torraccio</t>
+          <t>via_appia</t>
         </is>
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>gaz_torraccio</t>
+          <t>gaz_via_appia</t>
         </is>
       </c>
       <c r="E875" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I875" t="inlineStr">
@@ -37297,33 +37303,33 @@
         </is>
       </c>
       <c r="K875" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>interp_00875</t>
+          <t>interp_00877</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>ref_00688</t>
+          <t>ref_00689</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
         <is>
-          <t>torraccio</t>
+          <t>via_appia</t>
         </is>
       </c>
       <c r="D876" t="inlineStr">
         <is>
-          <t>gaz_torraccio</t>
+          <t>gaz_via_appia</t>
         </is>
       </c>
       <c r="E876" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I876" t="inlineStr">
@@ -37337,13 +37343,13 @@
         </is>
       </c>
       <c r="K876" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>interp_00876</t>
+          <t>interp_00878</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
@@ -37363,7 +37369,7 @@
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I877" t="inlineStr">
@@ -37383,7 +37389,7 @@
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>interp_00877</t>
+          <t>interp_00879</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
@@ -37403,7 +37409,7 @@
       </c>
       <c r="E878" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I878" t="inlineStr">
@@ -37423,27 +37429,27 @@
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>interp_00878</t>
+          <t>interp_00880</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>ref_00689</t>
+          <t>ref_00690</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>via_appia</t>
+          <t>due_santi</t>
         </is>
       </c>
       <c r="D879" t="inlineStr">
         <is>
-          <t>gaz_via_appia</t>
+          <t>gaz_due_santi</t>
         </is>
       </c>
       <c r="E879" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I879" t="inlineStr">
@@ -37457,33 +37463,33 @@
         </is>
       </c>
       <c r="K879" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>interp_00879</t>
+          <t>interp_00881</t>
         </is>
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>ref_00689</t>
+          <t>ref_00690</t>
         </is>
       </c>
       <c r="C880" t="inlineStr">
         <is>
-          <t>via_appia</t>
+          <t>due_santi</t>
         </is>
       </c>
       <c r="D880" t="inlineStr">
         <is>
-          <t>gaz_via_appia</t>
+          <t>gaz_due_santi</t>
         </is>
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I880" t="inlineStr">
@@ -37497,13 +37503,13 @@
         </is>
       </c>
       <c r="K880" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>interp_00880</t>
+          <t>interp_00882</t>
         </is>
       </c>
       <c r="B881" t="inlineStr">
@@ -37523,7 +37529,7 @@
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I881" t="inlineStr">
@@ -37543,7 +37549,7 @@
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>interp_00881</t>
+          <t>interp_00883</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
@@ -37563,7 +37569,7 @@
       </c>
       <c r="E882" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I882" t="inlineStr">
@@ -37583,27 +37589,27 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>interp_00882</t>
+          <t>interp_00884</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>ref_00690</t>
+          <t>ref_00691</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>due_santi</t>
+          <t>via_della_falcognana</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>gaz_due_santi</t>
+          <t>gaz_via_della_falcognana</t>
         </is>
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I883" t="inlineStr">
@@ -37617,33 +37623,33 @@
         </is>
       </c>
       <c r="K883" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>interp_00883</t>
+          <t>interp_00885</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>ref_00690</t>
+          <t>ref_00691</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>due_santi</t>
+          <t>via_della_falcognana</t>
         </is>
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>gaz_due_santi</t>
+          <t>gaz_via_della_falcognana</t>
         </is>
       </c>
       <c r="E884" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I884" t="inlineStr">
@@ -37657,13 +37663,13 @@
         </is>
       </c>
       <c r="K884" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>interp_00884</t>
+          <t>interp_00886</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
@@ -37683,7 +37689,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I885" t="inlineStr">
@@ -37703,7 +37709,7 @@
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>interp_00885</t>
+          <t>interp_00887</t>
         </is>
       </c>
       <c r="B886" t="inlineStr">
@@ -37723,7 +37729,7 @@
       </c>
       <c r="E886" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I886" t="inlineStr">
@@ -37743,27 +37749,27 @@
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>interp_00886</t>
+          <t>interp_00888</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>ref_00691</t>
+          <t>ref_00692</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>via_della_falcognana</t>
+          <t>via_anziate</t>
         </is>
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>gaz_via_della_falcognana</t>
+          <t>gaz_via_anziate</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I887" t="inlineStr">
@@ -37777,33 +37783,33 @@
         </is>
       </c>
       <c r="K887" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>interp_00887</t>
+          <t>interp_00889</t>
         </is>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>ref_00691</t>
+          <t>ref_00692</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>via_della_falcognana</t>
+          <t>via_anziate</t>
         </is>
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>gaz_via_della_falcognana</t>
+          <t>gaz_via_anziate</t>
         </is>
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I888" t="inlineStr">
@@ -37817,13 +37823,13 @@
         </is>
       </c>
       <c r="K888" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t>interp_00888</t>
+          <t>interp_00890</t>
         </is>
       </c>
       <c r="B889" t="inlineStr">
@@ -37843,7 +37849,7 @@
       </c>
       <c r="E889" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I889" t="inlineStr">
@@ -37863,7 +37869,7 @@
     <row r="890">
       <c r="A890" t="inlineStr">
         <is>
-          <t>interp_00889</t>
+          <t>interp_00891</t>
         </is>
       </c>
       <c r="B890" t="inlineStr">
@@ -37883,7 +37889,7 @@
       </c>
       <c r="E890" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I890" t="inlineStr">
@@ -37903,27 +37909,32 @@
     <row r="891">
       <c r="A891" t="inlineStr">
         <is>
-          <t>interp_00890</t>
+          <t>interp_00892</t>
         </is>
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>ref_00692</t>
+          <t>ref_00693</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>via_anziate</t>
+          <t>ponte_di_santa_fumia</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>gaz_via_anziate</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E891" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
       <c r="I891" t="inlineStr">
@@ -37937,33 +37948,38 @@
         </is>
       </c>
       <c r="K891" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>interp_00891</t>
+          <t>interp_00893</t>
         </is>
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>ref_00692</t>
+          <t>ref_00693</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>via_anziate</t>
+          <t>ponte_di_santa_fumia</t>
         </is>
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>gaz_via_anziate</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E892" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
       <c r="I892" t="inlineStr">
@@ -37977,13 +37993,13 @@
         </is>
       </c>
       <c r="K892" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
-          <t>interp_00892</t>
+          <t>interp_00894</t>
         </is>
       </c>
       <c r="B893" t="inlineStr">
@@ -38003,7 +38019,7 @@
       </c>
       <c r="E893" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="H893" t="inlineStr">
@@ -38028,7 +38044,7 @@
     <row r="894">
       <c r="A894" t="inlineStr">
         <is>
-          <t>interp_00893</t>
+          <t>interp_00895</t>
         </is>
       </c>
       <c r="B894" t="inlineStr">
@@ -38048,7 +38064,7 @@
       </c>
       <c r="E894" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="H894" t="inlineStr">
@@ -38073,17 +38089,17 @@
     <row r="895">
       <c r="A895" t="inlineStr">
         <is>
-          <t>interp_00894</t>
+          <t>interp_00896</t>
         </is>
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>ref_00693</t>
+          <t>ref_00694</t>
         </is>
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>ponte_di_santa_fumia</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
@@ -38093,12 +38109,12 @@
       </c>
       <c r="E895" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="H895" t="inlineStr">
         <is>
-          <t>inside</t>
+          <t>near</t>
         </is>
       </c>
       <c r="I895" t="inlineStr">
@@ -38112,23 +38128,23 @@
         </is>
       </c>
       <c r="K895" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="896">
       <c r="A896" t="inlineStr">
         <is>
-          <t>interp_00895</t>
+          <t>interp_00897</t>
         </is>
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>ref_00693</t>
+          <t>ref_00694</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>ponte_di_santa_fumia</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
@@ -38138,12 +38154,12 @@
       </c>
       <c r="E896" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="H896" t="inlineStr">
         <is>
-          <t>inside</t>
+          <t>near</t>
         </is>
       </c>
       <c r="I896" t="inlineStr">
@@ -38157,13 +38173,13 @@
         </is>
       </c>
       <c r="K896" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
         <is>
-          <t>interp_00896</t>
+          <t>interp_00898</t>
         </is>
       </c>
       <c r="B897" t="inlineStr">
@@ -38183,7 +38199,7 @@
       </c>
       <c r="E897" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="H897" t="inlineStr">
@@ -38208,7 +38224,7 @@
     <row r="898">
       <c r="A898" t="inlineStr">
         <is>
-          <t>interp_00897</t>
+          <t>interp_00899</t>
         </is>
       </c>
       <c r="B898" t="inlineStr">
@@ -38228,7 +38244,7 @@
       </c>
       <c r="E898" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="H898" t="inlineStr">
@@ -38253,32 +38269,27 @@
     <row r="899">
       <c r="A899" t="inlineStr">
         <is>
-          <t>interp_00898</t>
+          <t>interp_00900</t>
         </is>
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>ref_00694</t>
+          <t>ref_00695</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D899" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E899" t="inlineStr">
         <is>
-          <t>autista_questura</t>
-        </is>
-      </c>
-      <c r="H899" t="inlineStr">
-        <is>
-          <t>near</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I899" t="inlineStr">
@@ -38292,38 +38303,33 @@
         </is>
       </c>
       <c r="K899" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
         <is>
-          <t>interp_00899</t>
+          <t>interp_00901</t>
         </is>
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>ref_00694</t>
+          <t>ref_00695</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D900" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
-        </is>
-      </c>
-      <c r="H900" t="inlineStr">
-        <is>
-          <t>near</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I900" t="inlineStr">
@@ -38337,13 +38343,13 @@
         </is>
       </c>
       <c r="K900" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
         <is>
-          <t>interp_00900</t>
+          <t>interp_00902</t>
         </is>
       </c>
       <c r="B901" t="inlineStr">
@@ -38363,7 +38369,7 @@
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I901" t="inlineStr">
@@ -38383,7 +38389,7 @@
     <row r="902">
       <c r="A902" t="inlineStr">
         <is>
-          <t>interp_00901</t>
+          <t>interp_00903</t>
         </is>
       </c>
       <c r="B902" t="inlineStr">
@@ -38403,7 +38409,7 @@
       </c>
       <c r="E902" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I902" t="inlineStr">
@@ -38423,27 +38429,27 @@
     <row r="903">
       <c r="A903" t="inlineStr">
         <is>
-          <t>interp_00902</t>
+          <t>interp_00904</t>
         </is>
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>ref_00695</t>
+          <t>ref_00696</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>ferrovia_roma_velletri</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_ferrovia_roma_velletri</t>
         </is>
       </c>
       <c r="E903" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I903" t="inlineStr">
@@ -38457,33 +38463,33 @@
         </is>
       </c>
       <c r="K903" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>interp_00903</t>
+          <t>interp_00905</t>
         </is>
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>ref_00695</t>
+          <t>ref_00696</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>ferrovia_roma_velletri</t>
         </is>
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_ferrovia_roma_velletri</t>
         </is>
       </c>
       <c r="E904" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I904" t="inlineStr">
@@ -38497,13 +38503,13 @@
         </is>
       </c>
       <c r="K904" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" t="inlineStr">
         <is>
-          <t>interp_00904</t>
+          <t>interp_00906</t>
         </is>
       </c>
       <c r="B905" t="inlineStr">
@@ -38523,7 +38529,7 @@
       </c>
       <c r="E905" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I905" t="inlineStr">
@@ -38543,7 +38549,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>interp_00905</t>
+          <t>interp_00907</t>
         </is>
       </c>
       <c r="B906" t="inlineStr">
@@ -38563,7 +38569,7 @@
       </c>
       <c r="E906" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I906" t="inlineStr">
@@ -38583,27 +38589,27 @@
     <row r="907">
       <c r="A907" t="inlineStr">
         <is>
-          <t>interp_00906</t>
+          <t>interp_00908</t>
         </is>
       </c>
       <c r="B907" t="inlineStr">
         <is>
-          <t>ref_00696</t>
+          <t>ref_00697</t>
         </is>
       </c>
       <c r="C907" t="inlineStr">
         <is>
-          <t>ferrovia_roma_velletri</t>
+          <t>ponte_divino_amore</t>
         </is>
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>gaz_ferrovia_roma_velletri</t>
+          <t>gaz_ponte_divino_amore</t>
         </is>
       </c>
       <c r="E907" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="I907" t="inlineStr">
@@ -38617,33 +38623,33 @@
         </is>
       </c>
       <c r="K907" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="908">
       <c r="A908" t="inlineStr">
         <is>
-          <t>interp_00907</t>
+          <t>interp_00909</t>
         </is>
       </c>
       <c r="B908" t="inlineStr">
         <is>
-          <t>ref_00696</t>
+          <t>ref_00697</t>
         </is>
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>ferrovia_roma_velletri</t>
+          <t>ponte_divino_amore</t>
         </is>
       </c>
       <c r="D908" t="inlineStr">
         <is>
-          <t>gaz_ferrovia_roma_velletri</t>
+          <t>gaz_ponte_divino_amore</t>
         </is>
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="I908" t="inlineStr">
@@ -38657,13 +38663,13 @@
         </is>
       </c>
       <c r="K908" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
         <is>
-          <t>interp_00908</t>
+          <t>interp_00910</t>
         </is>
       </c>
       <c r="B909" t="inlineStr">
@@ -38683,7 +38689,7 @@
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="I909" t="inlineStr">
@@ -38703,7 +38709,7 @@
     <row r="910">
       <c r="A910" t="inlineStr">
         <is>
-          <t>interp_00909</t>
+          <t>interp_00911</t>
         </is>
       </c>
       <c r="B910" t="inlineStr">
@@ -38723,7 +38729,7 @@
       </c>
       <c r="E910" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="I910" t="inlineStr">
@@ -38743,87 +38749,71 @@
     <row r="911">
       <c r="A911" t="inlineStr">
         <is>
-          <t>interp_00910</t>
+          <t>interp_00912</t>
         </is>
       </c>
       <c r="B911" t="inlineStr">
         <is>
-          <t>ref_00697</t>
+          <t>ref_00698</t>
         </is>
       </c>
       <c r="C911" t="inlineStr">
         <is>
-          <t>ponte_divino_amore</t>
-        </is>
-      </c>
-      <c r="D911" t="inlineStr">
-        <is>
-          <t>gaz_ponte_divino_amore</t>
+          <t>tragitto_torraccio_ponte_divino_amore</t>
         </is>
       </c>
       <c r="E911" t="inlineStr">
         <is>
-          <t>autista_questura</t>
-        </is>
-      </c>
-      <c r="I911" t="inlineStr">
-        <is>
-          <t>routenode</t>
-        </is>
-      </c>
-      <c r="J911" t="inlineStr">
-        <is>
-          <t>tragitto_torraccio_ponte_divino_amore</t>
-        </is>
-      </c>
-      <c r="K911" t="n">
-        <v>10</v>
+          <t>ingravallo</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
       </c>
     </row>
     <row r="912">
       <c r="A912" t="inlineStr">
         <is>
-          <t>interp_00911</t>
+          <t>interp_00913</t>
         </is>
       </c>
       <c r="B912" t="inlineStr">
         <is>
-          <t>ref_00697</t>
+          <t>ref_00698</t>
         </is>
       </c>
       <c r="C912" t="inlineStr">
         <is>
-          <t>ponte_divino_amore</t>
-        </is>
-      </c>
-      <c r="D912" t="inlineStr">
-        <is>
-          <t>gaz_ponte_divino_amore</t>
+          <t>tragitto_torraccio_ponte_divino_amore</t>
         </is>
       </c>
       <c r="E912" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
-        </is>
-      </c>
-      <c r="I912" t="inlineStr">
-        <is>
-          <t>routenode</t>
-        </is>
-      </c>
-      <c r="J912" t="inlineStr">
-        <is>
-          <t>tragitto_torraccio_ponte_divino_amore</t>
-        </is>
-      </c>
-      <c r="K912" t="n">
-        <v>10</v>
+          <t>maresciallo_di_pietrantonio</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>approximate</t>
+        </is>
       </c>
     </row>
     <row r="913">
       <c r="A913" t="inlineStr">
         <is>
-          <t>interp_00912</t>
+          <t>interp_00914</t>
         </is>
       </c>
       <c r="B913" t="inlineStr">
@@ -38838,7 +38828,7 @@
       </c>
       <c r="E913" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>autista_questura</t>
         </is>
       </c>
       <c r="F913" t="inlineStr">
@@ -38855,7 +38845,7 @@
     <row r="914">
       <c r="A914" t="inlineStr">
         <is>
-          <t>interp_00913</t>
+          <t>interp_00915</t>
         </is>
       </c>
       <c r="B914" t="inlineStr">
@@ -38870,7 +38860,7 @@
       </c>
       <c r="E914" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="F914" t="inlineStr">
@@ -38887,59 +38877,74 @@
     <row r="915">
       <c r="A915" t="inlineStr">
         <is>
-          <t>interp_00914</t>
+          <t>interp_00916</t>
         </is>
       </c>
       <c r="B915" t="inlineStr">
         <is>
-          <t>ref_00698</t>
+          <t>ref_00699</t>
         </is>
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>tragitto_torraccio_ponte_divino_amore</t>
+          <t>tor_di_gheppio</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E915" t="inlineStr">
         <is>
-          <t>autista_questura</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F915" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G915" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="916">
       <c r="A916" t="inlineStr">
         <is>
-          <t>interp_00915</t>
+          <t>interp_00917</t>
         </is>
       </c>
       <c r="B916" t="inlineStr">
         <is>
-          <t>ref_00698</t>
+          <t>ref_00700</t>
         </is>
       </c>
       <c r="C916" t="inlineStr">
         <is>
-          <t>tragitto_torraccio_ponte_divino_amore</t>
+          <t>palazzo</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>gaz_palazzo</t>
         </is>
       </c>
       <c r="E916" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F916" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G916" t="inlineStr">
@@ -38951,74 +38956,69 @@
     <row r="917">
       <c r="A917" t="inlineStr">
         <is>
-          <t>interp_00916</t>
+          <t>interp_00918</t>
         </is>
       </c>
       <c r="B917" t="inlineStr">
         <is>
-          <t>ref_00699</t>
+          <t>ref_00701</t>
         </is>
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E917" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="F917" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G917" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H917" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="918">
       <c r="A918" t="inlineStr">
         <is>
-          <t>interp_00917</t>
+          <t>interp_00919</t>
         </is>
       </c>
       <c r="B918" t="inlineStr">
         <is>
-          <t>ref_00700</t>
+          <t>ref_00701</t>
         </is>
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>palazzo</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>gaz_palazzo</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E918" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F918" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>marker</t>
         </is>
       </c>
       <c r="G918" t="inlineStr">
@@ -39030,17 +39030,17 @@
     <row r="919">
       <c r="A919" t="inlineStr">
         <is>
-          <t>interp_00918</t>
+          <t>interp_00920</t>
         </is>
       </c>
       <c r="B919" t="inlineStr">
         <is>
-          <t>ref_00701</t>
+          <t>ref_00702</t>
         </is>
       </c>
       <c r="C919" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>stazione_pavona</t>
         </is>
       </c>
       <c r="D919" t="inlineStr">
@@ -39061,23 +39061,28 @@
       <c r="G919" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
         <is>
-          <t>interp_00919</t>
+          <t>interp_00921</t>
         </is>
       </c>
       <c r="B920" t="inlineStr">
         <is>
-          <t>ref_00701</t>
+          <t>ref_00702</t>
         </is>
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>stazione_pavona</t>
         </is>
       </c>
       <c r="D920" t="inlineStr">
@@ -39098,33 +39103,38 @@
       <c r="G920" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="921">
       <c r="A921" t="inlineStr">
         <is>
-          <t>interp_00920</t>
+          <t>interp_00922</t>
         </is>
       </c>
       <c r="B921" t="inlineStr">
         <is>
-          <t>ref_00702</t>
+          <t>ref_00703</t>
         </is>
       </c>
       <c r="C921" t="inlineStr">
         <is>
-          <t>stazione_pavona</t>
+          <t>direttissima_roma_napoli</t>
         </is>
       </c>
       <c r="D921" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_direttissima_roma_napoli</t>
         </is>
       </c>
       <c r="E921" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F921" t="inlineStr">
@@ -39135,38 +39145,33 @@
       <c r="G921" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H921" t="inlineStr">
-        <is>
-          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="922">
       <c r="A922" t="inlineStr">
         <is>
-          <t>interp_00921</t>
+          <t>interp_00923</t>
         </is>
       </c>
       <c r="B922" t="inlineStr">
         <is>
-          <t>ref_00702</t>
+          <t>ref_00703</t>
         </is>
       </c>
       <c r="C922" t="inlineStr">
         <is>
-          <t>stazione_pavona</t>
+          <t>direttissima_roma_napoli</t>
         </is>
       </c>
       <c r="D922" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_direttissima_roma_napoli</t>
         </is>
       </c>
       <c r="E922" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>agente_runzato</t>
         </is>
       </c>
       <c r="F922" t="inlineStr">
@@ -39177,33 +39182,28 @@
       <c r="G922" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H922" t="inlineStr">
-        <is>
-          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="inlineStr">
         <is>
-          <t>interp_00922</t>
+          <t>interp_00924</t>
         </is>
       </c>
       <c r="B923" t="inlineStr">
         <is>
-          <t>ref_00703</t>
+          <t>ref_00704</t>
         </is>
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>direttissima_roma_napoli</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D923" t="inlineStr">
         <is>
-          <t>gaz_direttissima_roma_napoli</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E923" t="inlineStr">
@@ -39213,34 +39213,39 @@
       </c>
       <c r="F923" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G923" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="inlineStr">
         <is>
-          <t>interp_00923</t>
+          <t>interp_00925</t>
         </is>
       </c>
       <c r="B924" t="inlineStr">
         <is>
-          <t>ref_00703</t>
+          <t>ref_00704</t>
         </is>
       </c>
       <c r="C924" t="inlineStr">
         <is>
-          <t>direttissima_roma_napoli</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D924" t="inlineStr">
         <is>
-          <t>gaz_direttissima_roma_napoli</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E924" t="inlineStr">
@@ -39250,34 +39255,39 @@
       </c>
       <c r="F924" t="inlineStr">
         <is>
-          <t>marker</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G924" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="925">
       <c r="A925" t="inlineStr">
         <is>
-          <t>interp_00924</t>
+          <t>interp_00926</t>
         </is>
       </c>
       <c r="B925" t="inlineStr">
         <is>
-          <t>ref_00704</t>
+          <t>ref_00705</t>
         </is>
       </c>
       <c r="C925" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D925" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E925" t="inlineStr">
@@ -39293,33 +39303,28 @@
       <c r="G925" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H925" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="926">
       <c r="A926" t="inlineStr">
         <is>
-          <t>interp_00925</t>
+          <t>interp_00927</t>
         </is>
       </c>
       <c r="B926" t="inlineStr">
         <is>
-          <t>ref_00704</t>
+          <t>ref_00705</t>
         </is>
       </c>
       <c r="C926" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D926" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E926" t="inlineStr">
@@ -39335,33 +39340,28 @@
       <c r="G926" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H926" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
         <is>
-          <t>interp_00926</t>
+          <t>interp_00928</t>
         </is>
       </c>
       <c r="B927" t="inlineStr">
         <is>
-          <t>ref_00705</t>
+          <t>ref_00706</t>
         </is>
       </c>
       <c r="C927" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D927" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E927" t="inlineStr">
@@ -39383,22 +39383,22 @@
     <row r="928">
       <c r="A928" t="inlineStr">
         <is>
-          <t>interp_00927</t>
+          <t>interp_00929</t>
         </is>
       </c>
       <c r="B928" t="inlineStr">
         <is>
-          <t>ref_00705</t>
+          <t>ref_00706</t>
         </is>
       </c>
       <c r="C928" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D928" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E928" t="inlineStr">
@@ -39420,22 +39420,22 @@
     <row r="929">
       <c r="A929" t="inlineStr">
         <is>
-          <t>interp_00928</t>
+          <t>interp_00930</t>
         </is>
       </c>
       <c r="B929" t="inlineStr">
         <is>
-          <t>ref_00706</t>
+          <t>ref_00707</t>
         </is>
       </c>
       <c r="C929" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>via_ardeatina</t>
         </is>
       </c>
       <c r="D929" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_via_ardeatina</t>
         </is>
       </c>
       <c r="E929" t="inlineStr">
@@ -39457,22 +39457,22 @@
     <row r="930">
       <c r="A930" t="inlineStr">
         <is>
-          <t>interp_00929</t>
+          <t>interp_00931</t>
         </is>
       </c>
       <c r="B930" t="inlineStr">
         <is>
-          <t>ref_00706</t>
+          <t>ref_00707</t>
         </is>
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>via_ardeatina</t>
         </is>
       </c>
       <c r="D930" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_via_ardeatina</t>
         </is>
       </c>
       <c r="E930" t="inlineStr">
@@ -39494,22 +39494,22 @@
     <row r="931">
       <c r="A931" t="inlineStr">
         <is>
-          <t>interp_00930</t>
+          <t>interp_00932</t>
         </is>
       </c>
       <c r="B931" t="inlineStr">
         <is>
-          <t>ref_00707</t>
+          <t>ref_00708</t>
         </is>
       </c>
       <c r="C931" t="inlineStr">
         <is>
-          <t>via_ardeatina</t>
+          <t>ardea</t>
         </is>
       </c>
       <c r="D931" t="inlineStr">
         <is>
-          <t>gaz_via_ardeatina</t>
+          <t>gaz_ardea</t>
         </is>
       </c>
       <c r="E931" t="inlineStr">
@@ -39531,22 +39531,22 @@
     <row r="932">
       <c r="A932" t="inlineStr">
         <is>
-          <t>interp_00931</t>
+          <t>interp_00933</t>
         </is>
       </c>
       <c r="B932" t="inlineStr">
         <is>
-          <t>ref_00707</t>
+          <t>ref_00708</t>
         </is>
       </c>
       <c r="C932" t="inlineStr">
         <is>
-          <t>via_ardeatina</t>
+          <t>ardea</t>
         </is>
       </c>
       <c r="D932" t="inlineStr">
         <is>
-          <t>gaz_via_ardeatina</t>
+          <t>gaz_ardea</t>
         </is>
       </c>
       <c r="E932" t="inlineStr">
@@ -39568,22 +39568,22 @@
     <row r="933">
       <c r="A933" t="inlineStr">
         <is>
-          <t>interp_00932</t>
+          <t>interp_00934</t>
         </is>
       </c>
       <c r="B933" t="inlineStr">
         <is>
-          <t>ref_00708</t>
+          <t>ref_00709</t>
         </is>
       </c>
       <c r="C933" t="inlineStr">
         <is>
-          <t>ardea</t>
+          <t>santa_palomba</t>
         </is>
       </c>
       <c r="D933" t="inlineStr">
         <is>
-          <t>gaz_ardea</t>
+          <t>gaz_santa_palomba</t>
         </is>
       </c>
       <c r="E933" t="inlineStr">
@@ -39605,22 +39605,22 @@
     <row r="934">
       <c r="A934" t="inlineStr">
         <is>
-          <t>interp_00933</t>
+          <t>interp_00935</t>
         </is>
       </c>
       <c r="B934" t="inlineStr">
         <is>
-          <t>ref_00708</t>
+          <t>ref_00709</t>
         </is>
       </c>
       <c r="C934" t="inlineStr">
         <is>
-          <t>ardea</t>
+          <t>santa_palomba</t>
         </is>
       </c>
       <c r="D934" t="inlineStr">
         <is>
-          <t>gaz_ardea</t>
+          <t>gaz_santa_palomba</t>
         </is>
       </c>
       <c r="E934" t="inlineStr">
@@ -39642,22 +39642,22 @@
     <row r="935">
       <c r="A935" t="inlineStr">
         <is>
-          <t>interp_00934</t>
+          <t>interp_00936</t>
         </is>
       </c>
       <c r="B935" t="inlineStr">
         <is>
-          <t>ref_00709</t>
+          <t>ref_00710</t>
         </is>
       </c>
       <c r="C935" t="inlineStr">
         <is>
-          <t>santa_palomba</t>
+          <t>marino</t>
         </is>
       </c>
       <c r="D935" t="inlineStr">
         <is>
-          <t>gaz_santa_palomba</t>
+          <t>gaz_marino</t>
         </is>
       </c>
       <c r="E935" t="inlineStr">
@@ -39679,22 +39679,22 @@
     <row r="936">
       <c r="A936" t="inlineStr">
         <is>
-          <t>interp_00935</t>
+          <t>interp_00937</t>
         </is>
       </c>
       <c r="B936" t="inlineStr">
         <is>
-          <t>ref_00709</t>
+          <t>ref_00710</t>
         </is>
       </c>
       <c r="C936" t="inlineStr">
         <is>
-          <t>santa_palomba</t>
+          <t>marino</t>
         </is>
       </c>
       <c r="D936" t="inlineStr">
         <is>
-          <t>gaz_santa_palomba</t>
+          <t>gaz_marino</t>
         </is>
       </c>
       <c r="E936" t="inlineStr">
@@ -39716,22 +39716,22 @@
     <row r="937">
       <c r="A937" t="inlineStr">
         <is>
-          <t>interp_00936</t>
+          <t>interp_00938</t>
         </is>
       </c>
       <c r="B937" t="inlineStr">
         <is>
-          <t>ref_00710</t>
+          <t>ref_00711</t>
         </is>
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>marino</t>
+          <t>solforata</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>gaz_marino</t>
+          <t>gaz_solforata</t>
         </is>
       </c>
       <c r="E937" t="inlineStr">
@@ -39753,22 +39753,22 @@
     <row r="938">
       <c r="A938" t="inlineStr">
         <is>
-          <t>interp_00937</t>
+          <t>interp_00939</t>
         </is>
       </c>
       <c r="B938" t="inlineStr">
         <is>
-          <t>ref_00710</t>
+          <t>ref_00711</t>
         </is>
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>marino</t>
+          <t>solforata</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>gaz_marino</t>
+          <t>gaz_solforata</t>
         </is>
       </c>
       <c r="E938" t="inlineStr">
@@ -39790,22 +39790,22 @@
     <row r="939">
       <c r="A939" t="inlineStr">
         <is>
-          <t>interp_00938</t>
+          <t>interp_00940</t>
         </is>
       </c>
       <c r="B939" t="inlineStr">
         <is>
-          <t>ref_00711</t>
+          <t>ref_00712</t>
         </is>
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>solforata</t>
+          <t>pratica_di_mare</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>gaz_solforata</t>
+          <t>gaz_pratica_di_mare</t>
         </is>
       </c>
       <c r="E939" t="inlineStr">
@@ -39827,22 +39827,22 @@
     <row r="940">
       <c r="A940" t="inlineStr">
         <is>
-          <t>interp_00939</t>
+          <t>interp_00941</t>
         </is>
       </c>
       <c r="B940" t="inlineStr">
         <is>
-          <t>ref_00711</t>
+          <t>ref_00712</t>
         </is>
       </c>
       <c r="C940" t="inlineStr">
         <is>
-          <t>solforata</t>
+          <t>pratica_di_mare</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>gaz_solforata</t>
+          <t>gaz_pratica_di_mare</t>
         </is>
       </c>
       <c r="E940" t="inlineStr">
@@ -39864,22 +39864,22 @@
     <row r="941">
       <c r="A941" t="inlineStr">
         <is>
-          <t>interp_00940</t>
+          <t>interp_00942</t>
         </is>
       </c>
       <c r="B941" t="inlineStr">
         <is>
-          <t>ref_00712</t>
+          <t>ref_00713</t>
         </is>
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>pratica_di_mare</t>
+          <t>palazzo</t>
         </is>
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>gaz_pratica_di_mare</t>
+          <t>gaz_palazzo</t>
         </is>
       </c>
       <c r="E941" t="inlineStr">
@@ -39901,22 +39901,22 @@
     <row r="942">
       <c r="A942" t="inlineStr">
         <is>
-          <t>interp_00941</t>
+          <t>interp_00943</t>
         </is>
       </c>
       <c r="B942" t="inlineStr">
         <is>
-          <t>ref_00712</t>
+          <t>ref_00713</t>
         </is>
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>pratica_di_mare</t>
+          <t>palazzo</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>gaz_pratica_di_mare</t>
+          <t>gaz_palazzo</t>
         </is>
       </c>
       <c r="E942" t="inlineStr">
@@ -39938,22 +39938,22 @@
     <row r="943">
       <c r="A943" t="inlineStr">
         <is>
-          <t>interp_00942</t>
+          <t>interp_00944</t>
         </is>
       </c>
       <c r="B943" t="inlineStr">
         <is>
-          <t>ref_00713</t>
+          <t>ref_00714</t>
         </is>
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>palazzo</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>gaz_palazzo</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E943" t="inlineStr">
@@ -39975,22 +39975,22 @@
     <row r="944">
       <c r="A944" t="inlineStr">
         <is>
-          <t>interp_00943</t>
+          <t>interp_00945</t>
         </is>
       </c>
       <c r="B944" t="inlineStr">
         <is>
-          <t>ref_00713</t>
+          <t>ref_00714</t>
         </is>
       </c>
       <c r="C944" t="inlineStr">
         <is>
-          <t>palazzo</t>
+          <t>pavona</t>
         </is>
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>gaz_palazzo</t>
+          <t>gaz_pavona</t>
         </is>
       </c>
       <c r="E944" t="inlineStr">
@@ -40012,22 +40012,22 @@
     <row r="945">
       <c r="A945" t="inlineStr">
         <is>
-          <t>interp_00944</t>
+          <t>interp_00946</t>
         </is>
       </c>
       <c r="B945" t="inlineStr">
         <is>
-          <t>ref_00714</t>
+          <t>ref_00715</t>
         </is>
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E945" t="inlineStr">
@@ -40049,22 +40049,22 @@
     <row r="946">
       <c r="A946" t="inlineStr">
         <is>
-          <t>interp_00945</t>
+          <t>interp_00947</t>
         </is>
       </c>
       <c r="B946" t="inlineStr">
         <is>
-          <t>ref_00714</t>
+          <t>ref_00715</t>
         </is>
       </c>
       <c r="C946" t="inlineStr">
         <is>
-          <t>pavona</t>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="D946" t="inlineStr">
         <is>
-          <t>gaz_pavona</t>
+          <t>gaz_casal_bruciato</t>
         </is>
       </c>
       <c r="E946" t="inlineStr">
@@ -40086,22 +40086,22 @@
     <row r="947">
       <c r="A947" t="inlineStr">
         <is>
-          <t>interp_00946</t>
+          <t>interp_00948</t>
         </is>
       </c>
       <c r="B947" t="inlineStr">
         <is>
-          <t>ref_00715</t>
+          <t>ref_00716</t>
         </is>
       </c>
       <c r="C947" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
@@ -40117,28 +40117,33 @@
       <c r="G947" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="948">
       <c r="A948" t="inlineStr">
         <is>
-          <t>interp_00947</t>
+          <t>interp_00949</t>
         </is>
       </c>
       <c r="B948" t="inlineStr">
         <is>
-          <t>ref_00715</t>
+          <t>ref_00716</t>
         </is>
       </c>
       <c r="C948" t="inlineStr">
         <is>
-          <t>casal_bruciato</t>
+          <t>tor_di_gheppio</t>
         </is>
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>gaz_casal_bruciato</t>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
@@ -40154,28 +40159,28 @@
       <c r="G948" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="949">
       <c r="A949" t="inlineStr">
         <is>
-          <t>interp_00948</t>
+          <t>interp_00950</t>
         </is>
       </c>
       <c r="B949" t="inlineStr">
         <is>
-          <t>ref_00716</t>
+          <t>ref_00717</t>
         </is>
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
-        </is>
-      </c>
-      <c r="D949" t="inlineStr">
-        <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>casa_crocchiapani</t>
         </is>
       </c>
       <c r="E949" t="inlineStr">
@@ -40185,39 +40190,29 @@
       </c>
       <c r="F949" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G949" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H949" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="950">
       <c r="A950" t="inlineStr">
         <is>
-          <t>interp_00949</t>
+          <t>interp_00951</t>
         </is>
       </c>
       <c r="B950" t="inlineStr">
         <is>
-          <t>ref_00716</t>
+          <t>ref_00717</t>
         </is>
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
-        </is>
-      </c>
-      <c r="D950" t="inlineStr">
-        <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>casa_crocchiapani</t>
         </is>
       </c>
       <c r="E950" t="inlineStr">
@@ -40227,24 +40222,19 @@
       </c>
       <c r="F950" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G950" t="inlineStr">
         <is>
           <t>approximate</t>
-        </is>
-      </c>
-      <c r="H950" t="inlineStr">
-        <is>
-          <t>near</t>
         </is>
       </c>
     </row>
     <row r="951">
       <c r="A951" t="inlineStr">
         <is>
-          <t>interp_00950</t>
+          <t>interp_00952</t>
         </is>
       </c>
       <c r="B951" t="inlineStr">
@@ -40259,7 +40249,7 @@
       </c>
       <c r="E951" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="F951" t="inlineStr">
@@ -40276,7 +40266,7 @@
     <row r="952">
       <c r="A952" t="inlineStr">
         <is>
-          <t>interp_00951</t>
+          <t>interp_00953</t>
         </is>
       </c>
       <c r="B952" t="inlineStr">
@@ -40291,7 +40281,7 @@
       </c>
       <c r="E952" t="inlineStr">
         <is>
-          <t>agente_runzato</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F952" t="inlineStr">
@@ -40308,12 +40298,12 @@
     <row r="953">
       <c r="A953" t="inlineStr">
         <is>
-          <t>interp_00952</t>
+          <t>interp_00954</t>
         </is>
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>ref_00717</t>
+          <t>ref_00718</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
@@ -40323,7 +40313,7 @@
       </c>
       <c r="E953" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F953" t="inlineStr">
@@ -40333,51 +40323,61 @@
       </c>
       <c r="G953" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>precise</t>
         </is>
       </c>
     </row>
     <row r="954">
       <c r="A954" t="inlineStr">
         <is>
-          <t>interp_00953</t>
+          <t>interp_00955</t>
         </is>
       </c>
       <c r="B954" t="inlineStr">
         <is>
-          <t>ref_00717</t>
+          <t>ref_00719</t>
         </is>
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>casa_crocchiapani</t>
+          <t>tor_di_gheppio</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E954" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>veronica_magliarini</t>
         </is>
       </c>
       <c r="F954" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G954" t="inlineStr">
         <is>
           <t>approximate</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="955">
       <c r="A955" t="inlineStr">
         <is>
-          <t>interp_00954</t>
+          <t>interp_00956</t>
         </is>
       </c>
       <c r="B955" t="inlineStr">
         <is>
-          <t>ref_00718</t>
+          <t>ref_00720</t>
         </is>
       </c>
       <c r="C955" t="inlineStr">
@@ -40387,7 +40387,7 @@
       </c>
       <c r="E955" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F955" t="inlineStr">
@@ -40404,49 +40404,39 @@
     <row r="956">
       <c r="A956" t="inlineStr">
         <is>
-          <t>interp_00955</t>
+          <t>interp_00957</t>
         </is>
       </c>
       <c r="B956" t="inlineStr">
         <is>
-          <t>ref_00719</t>
+          <t>ref_00720</t>
         </is>
       </c>
       <c r="C956" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
-        </is>
-      </c>
-      <c r="D956" t="inlineStr">
-        <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>casa_crocchiapani</t>
         </is>
       </c>
       <c r="E956" t="inlineStr">
         <is>
-          <t>veronica_magliarini</t>
+          <t>maresciallo_di_pietrantonio</t>
         </is>
       </c>
       <c r="F956" t="inlineStr">
         <is>
-          <t>projectedspace</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="G956" t="inlineStr">
         <is>
-          <t>approximate</t>
-        </is>
-      </c>
-      <c r="H956" t="inlineStr">
-        <is>
-          <t>near</t>
+          <t>precise</t>
         </is>
       </c>
     </row>
     <row r="957">
       <c r="A957" t="inlineStr">
         <is>
-          <t>interp_00956</t>
+          <t>interp_00958</t>
         </is>
       </c>
       <c r="B957" t="inlineStr">
@@ -40461,7 +40451,7 @@
       </c>
       <c r="E957" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F957" t="inlineStr">
@@ -40478,49 +40468,64 @@
     <row r="958">
       <c r="A958" t="inlineStr">
         <is>
-          <t>interp_00957</t>
+          <t>interp_00959</t>
         </is>
       </c>
       <c r="B958" t="inlineStr">
         <is>
-          <t>ref_00720</t>
+          <t>ref_00721</t>
         </is>
       </c>
       <c r="C958" t="inlineStr">
         <is>
-          <t>casa_crocchiapani</t>
+          <t>tor_di_gheppio</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E958" t="inlineStr">
         <is>
-          <t>maresciallo_di_pietrantonio</t>
+          <t>ingravallo</t>
         </is>
       </c>
       <c r="F958" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G958" t="inlineStr">
         <is>
-          <t>precise</t>
+          <t>relative</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="959">
       <c r="A959" t="inlineStr">
         <is>
-          <t>interp_00958</t>
+          <t>interp_00960</t>
         </is>
       </c>
       <c r="B959" t="inlineStr">
         <is>
-          <t>ref_00720</t>
+          <t>ref_00721</t>
         </is>
       </c>
       <c r="C959" t="inlineStr">
         <is>
-          <t>casa_crocchiapani</t>
+          <t>tor_di_gheppio</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>gaz_quarto_di_santa_fumia</t>
         </is>
       </c>
       <c r="E959" t="inlineStr">
@@ -40530,39 +40535,44 @@
       </c>
       <c r="F959" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G959" t="inlineStr">
         <is>
-          <t>precise</t>
+          <t>relative</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>near</t>
         </is>
       </c>
     </row>
     <row r="960">
       <c r="A960" t="inlineStr">
         <is>
-          <t>interp_00959</t>
+          <t>interp_00961</t>
         </is>
       </c>
       <c r="B960" t="inlineStr">
         <is>
-          <t>ref_00721</t>
+          <t>ref_00722</t>
         </is>
       </c>
       <c r="C960" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>tenenza_carabinieri_marino</t>
         </is>
       </c>
       <c r="D960" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_marino</t>
         </is>
       </c>
       <c r="E960" t="inlineStr">
         <is>
-          <t>ingravallo</t>
+          <t>assunta</t>
         </is>
       </c>
       <c r="F960" t="inlineStr">
@@ -40577,34 +40587,34 @@
       </c>
       <c r="H960" t="inlineStr">
         <is>
-          <t>near</t>
+          <t>inside</t>
         </is>
       </c>
     </row>
     <row r="961">
       <c r="A961" t="inlineStr">
         <is>
-          <t>interp_00960</t>
+          <t>interp_00962</t>
         </is>
       </c>
       <c r="B961" t="inlineStr">
         <is>
-          <t>ref_00721</t>
+          <t>ref_00722</t>
         </is>
       </c>
       <c r="C961" t="inlineStr">
         <is>
-          <t>tor_di_gheppio</t>
+          <t>tenenza_carabinieri_marino</t>
         </is>
       </c>
       <c r="D961" t="inlineStr">
         <is>
-          <t>gaz_quarto_di_santa_fumia</t>
+          <t>gaz_marino</t>
         </is>
       </c>
       <c r="E961" t="inlineStr">
         <is>
-          <t>assunta</t>
+          <t>pestalozzi</t>
         </is>
       </c>
       <c r="F961" t="inlineStr">
@@ -40618,90 +40628,6 @@
         </is>
       </c>
       <c r="H961" t="inlineStr">
-        <is>
-          <t>near</t>
-        </is>
-      </c>
-    </row>
-    <row r="962">
-      <c r="A962" t="inlineStr">
-        <is>
-          <t>interp_00961</t>
-        </is>
-      </c>
-      <c r="B962" t="inlineStr">
-        <is>
-          <t>ref_00722</t>
-        </is>
-      </c>
-      <c r="C962" t="inlineStr">
-        <is>
-          <t>tenenza_carabinieri_marino</t>
-        </is>
-      </c>
-      <c r="D962" t="inlineStr">
-        <is>
-          <t>gaz_marino</t>
-        </is>
-      </c>
-      <c r="E962" t="inlineStr">
-        <is>
-          <t>assunta</t>
-        </is>
-      </c>
-      <c r="F962" t="inlineStr">
-        <is>
-          <t>projectedspace</t>
-        </is>
-      </c>
-      <c r="G962" t="inlineStr">
-        <is>
-          <t>relative</t>
-        </is>
-      </c>
-      <c r="H962" t="inlineStr">
-        <is>
-          <t>inside</t>
-        </is>
-      </c>
-    </row>
-    <row r="963">
-      <c r="A963" t="inlineStr">
-        <is>
-          <t>interp_00962</t>
-        </is>
-      </c>
-      <c r="B963" t="inlineStr">
-        <is>
-          <t>ref_00722</t>
-        </is>
-      </c>
-      <c r="C963" t="inlineStr">
-        <is>
-          <t>tenenza_carabinieri_marino</t>
-        </is>
-      </c>
-      <c r="D963" t="inlineStr">
-        <is>
-          <t>gaz_marino</t>
-        </is>
-      </c>
-      <c r="E963" t="inlineStr">
-        <is>
-          <t>pestalozzi</t>
-        </is>
-      </c>
-      <c r="F963" t="inlineStr">
-        <is>
-          <t>projectedspace</t>
-        </is>
-      </c>
-      <c r="G963" t="inlineStr">
-        <is>
-          <t>relative</t>
-        </is>
-      </c>
-      <c r="H963" t="inlineStr">
         <is>
           <t>inside</t>
         </is>

</xml_diff>

<commit_message>
soglia, frontalità, confine; edicola adiacente all'orto (T-53, D-058)
Threshold, Facing, Boundary nello schema delle relazioni; il termine di un
ancoraggio relazionale può essere un luogo narrativo (relazione senza
referente, R17). Edicola ai Due Santi AdjacentTo orto/vigna (QP 216).
TBox 1.187 -> 1.217, ABox 27.144 -> 27.148, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/SpatialInterpretations.xlsx
+++ b/data/source/xlsx/SpatialInterpretations.xlsx
@@ -31591,6 +31591,16 @@
           <t>lorenzo_sabatino</t>
         </is>
       </c>
+      <c r="R660" t="inlineStr">
+        <is>
+          <t>orto_vigna_due_santi</t>
+        </is>
+      </c>
+      <c r="S660" t="inlineStr">
+        <is>
+          <t>adjacentto</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">

</xml_diff>

<commit_message>
Fase 3c: correzioni prima del merge (D-091)
Tolta interp_00973 (QPa 169, agente anonimo non registrato); below verso
il laboratorio spostato da QPa 165 a QPa 169; estratto di QPa 166 accorciato.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/SpatialInterpretations.xlsx
+++ b/data/source/xlsx/SpatialInterpretations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X970"/>
+  <dimension ref="A1:X969"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49659,7 +49659,7 @@
       </c>
       <c r="G960" t="inlineStr">
         <is>
-          <t>relative</t>
+          <t>approximate</t>
         </is>
       </c>
       <c r="H960" t="inlineStr">
@@ -49680,21 +49680,6 @@
       <c r="O960" t="inlineStr">
         <is>
           <t>close_reading</t>
-        </is>
-      </c>
-      <c r="P960" t="inlineStr">
-        <is>
-          <t>Il passo colloca la cantina «sotto al laboratorio-bettola» (QPa 165): relazione verticale con il laboratorio, dichiarata qui perché la frase non è nell'estratto (D-091).</t>
-        </is>
-      </c>
-      <c r="R960" t="inlineStr">
-        <is>
-          <t>laboratorio_zamira</t>
-        </is>
-      </c>
-      <c r="S960" t="inlineStr">
-        <is>
-          <t>below</t>
         </is>
       </c>
       <c r="T960" t="inlineStr">
@@ -49940,6 +49925,21 @@
           <t>close_reading</t>
         </is>
       </c>
+      <c r="P964" t="inlineStr">
+        <is>
+          <t>La Zamira manda a «levarseli in cantina» e a portare i pantaloni «su […] in laboratorio» (QPa 169): la cantina sta sotto il laboratorio (D-091).</t>
+        </is>
+      </c>
+      <c r="R964" t="inlineStr">
+        <is>
+          <t>laboratorio_zamira</t>
+        </is>
+      </c>
+      <c r="S964" t="inlineStr">
+        <is>
+          <t>below</t>
+        </is>
+      </c>
       <c r="T964" t="inlineStr">
         <is>
           <t>si</t>
@@ -49949,12 +49949,12 @@
     <row r="965">
       <c r="A965" t="inlineStr">
         <is>
-          <t>interp_00973</t>
+          <t>interp_00974</t>
         </is>
       </c>
       <c r="B965" t="inlineStr">
         <is>
-          <t>ref_00741</t>
+          <t>ref_00742</t>
         </is>
       </c>
       <c r="C965" t="inlineStr">
@@ -49964,17 +49964,17 @@
       </c>
       <c r="E965" t="inlineStr">
         <is>
-          <t>santarella</t>
+          <t>zamira_pacori</t>
         </is>
       </c>
       <c r="F965" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>projectedspace</t>
         </is>
       </c>
       <c r="G965" t="inlineStr">
         <is>
-          <t>relative</t>
+          <t>approximate</t>
         </is>
       </c>
       <c r="H965" t="inlineStr">
@@ -50006,7 +50006,7 @@
     <row r="966">
       <c r="A966" t="inlineStr">
         <is>
-          <t>interp_00974</t>
+          <t>interp_00975</t>
         </is>
       </c>
       <c r="B966" t="inlineStr">
@@ -50021,7 +50021,7 @@
       </c>
       <c r="E966" t="inlineStr">
         <is>
-          <t>zamira_pacori</t>
+          <t>diomede</t>
         </is>
       </c>
       <c r="F966" t="inlineStr">
@@ -50063,12 +50063,12 @@
     <row r="967">
       <c r="A967" t="inlineStr">
         <is>
-          <t>interp_00975</t>
+          <t>interp_00976</t>
         </is>
       </c>
       <c r="B967" t="inlineStr">
         <is>
-          <t>ref_00742</t>
+          <t>ref_00743</t>
         </is>
       </c>
       <c r="C967" t="inlineStr">
@@ -50078,7 +50078,7 @@
       </c>
       <c r="E967" t="inlineStr">
         <is>
-          <t>diomede</t>
+          <t>zamira_pacori</t>
         </is>
       </c>
       <c r="F967" t="inlineStr">
@@ -50088,7 +50088,7 @@
       </c>
       <c r="G967" t="inlineStr">
         <is>
-          <t>approximate</t>
+          <t>indeterminate</t>
         </is>
       </c>
       <c r="H967" t="inlineStr">
@@ -50120,7 +50120,7 @@
     <row r="968">
       <c r="A968" t="inlineStr">
         <is>
-          <t>interp_00976</t>
+          <t>interp_00977</t>
         </is>
       </c>
       <c r="B968" t="inlineStr">
@@ -50135,7 +50135,7 @@
       </c>
       <c r="E968" t="inlineStr">
         <is>
-          <t>zamira_pacori</t>
+          <t>diomede</t>
         </is>
       </c>
       <c r="F968" t="inlineStr">
@@ -50177,22 +50177,27 @@
     <row r="969">
       <c r="A969" t="inlineStr">
         <is>
-          <t>interp_00977</t>
+          <t>interp_00978</t>
         </is>
       </c>
       <c r="B969" t="inlineStr">
         <is>
-          <t>ref_00743</t>
+          <t>ref_00744</t>
         </is>
       </c>
       <c r="C969" t="inlineStr">
         <is>
-          <t>cantina_zamira</t>
+          <t>camera_sicurezza_questura</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>gaz_santo_stefano_del_cacco_celio_santo_stefano</t>
         </is>
       </c>
       <c r="E969" t="inlineStr">
         <is>
-          <t>diomede</t>
+          <t>ines_cionini</t>
         </is>
       </c>
       <c r="F969" t="inlineStr">
@@ -50202,7 +50207,7 @@
       </c>
       <c r="G969" t="inlineStr">
         <is>
-          <t>indeterminate</t>
+          <t>approximate</t>
         </is>
       </c>
       <c r="H969" t="inlineStr">
@@ -50226,68 +50231,6 @@
         </is>
       </c>
       <c r="T969" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-    </row>
-    <row r="970">
-      <c r="A970" t="inlineStr">
-        <is>
-          <t>interp_00978</t>
-        </is>
-      </c>
-      <c r="B970" t="inlineStr">
-        <is>
-          <t>ref_00744</t>
-        </is>
-      </c>
-      <c r="C970" t="inlineStr">
-        <is>
-          <t>camera_sicurezza_questura</t>
-        </is>
-      </c>
-      <c r="D970" t="inlineStr">
-        <is>
-          <t>gaz_santo_stefano_del_cacco_celio_santo_stefano</t>
-        </is>
-      </c>
-      <c r="E970" t="inlineStr">
-        <is>
-          <t>ines_cionini</t>
-        </is>
-      </c>
-      <c r="F970" t="inlineStr">
-        <is>
-          <t>projectedspace</t>
-        </is>
-      </c>
-      <c r="G970" t="inlineStr">
-        <is>
-          <t>approximate</t>
-        </is>
-      </c>
-      <c r="H970" t="inlineStr">
-        <is>
-          <t>inside</t>
-        </is>
-      </c>
-      <c r="M970" t="inlineStr">
-        <is>
-          <t>lorenzo_sabatino</t>
-        </is>
-      </c>
-      <c r="N970" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="O970" t="inlineStr">
-        <is>
-          <t>close_reading</t>
-        </is>
-      </c>
-      <c r="T970" t="inlineStr">
         <is>
           <t>si</t>
         </is>

</xml_diff>